<commit_message>
Fix ability type of Pugnacious Amphiptere and Sagacious Spitter
Both fledglings have a 'When Activated' (Adventurer) ability, not a
'When Played' one. Update the source spreadsheet and regenerate
cards.json.

Fixes #4
</commit_message>
<xml_diff>
--- a/scripts/cards.xlsx
+++ b/scripts/cards.xlsx
@@ -11322,7 +11322,7 @@
         <v>426</v>
       </c>
       <c r="E262" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="F262">
         <v>1</v>
@@ -11360,7 +11360,7 @@
         <v>428</v>
       </c>
       <c r="E263" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="F263">
         <v>1</v>

</xml_diff>